<commit_message>
Fix: Reparatur-Dialog behoben - ungueltige Formeln in bedingter Formatierung
Ursache: Die bedingte Formatierung enthielt noch deutsche Funktionsnamen
(HEUTE) und Semikolons. Excel speichert auch Formatierungs-Formeln intern
englisch mit Kommas, wodurch die Datei als beschaedigt gemeldet wurde.

- Bedingte Formatierung auf TODAY() und Komma-Trennung umgestellt
- Dashboard 'Naechste Meilensteine' von Matrixformel auf robuste
  AGGREGATE-Formel mit festen Bereichen umgestellt (kein CSE noetig)
- XML-Validierung: keine deutschen Funktionsnamen, keine Semikolons,
  alle Teile wohlgeformt, Tabellenspalten eindeutig

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YMxj9pzhuMuXneYjMXFmRT
</commit_message>
<xml_diff>
--- a/Projektsteuerung_MiT-PWR-WIN-2026-001.xlsx
+++ b/Projektsteuerung_MiT-PWR-WIN-2026-001.xlsx
@@ -1040,46 +1040,46 @@
     </row>
     <row r="18">
       <c r="B18" s="18">
-        <f t="array" ref="B18">IFERROR(SMALL(IF((Meilensteine[Status]&lt;&gt;"erledigt")*(Meilensteine[Plantermin]&gt;=TODAY()),Meilensteine[Plantermin]),1),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,Meilensteine!$C$2:$C$17/((Meilensteine!$E$2:$E$17&lt;&gt;"erledigt")*(Meilensteine!$C$2:$C$17&gt;=TODAY())),1),"")</f>
         <v/>
       </c>
       <c r="C18" s="4">
-        <f>IFERROR(INDEX(Meilensteine[Meilenstein],MATCH(B18,Meilensteine[Plantermin],0)),"")</f>
+        <f>IFERROR(INDEX(Meilensteine!$B$2:$B$17,MATCH(B18,Meilensteine!$C$2:$C$17,0)),"")</f>
         <v/>
       </c>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="19">
-        <f>IFERROR(INDEX(Meilensteine[Status],MATCH(B18,Meilensteine[Plantermin],0)),"")</f>
+        <f>IFERROR(INDEX(Meilensteine!$E$2:$E$17,MATCH(B18,Meilensteine!$C$2:$C$17,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="18">
-        <f t="array" ref="B19">IFERROR(SMALL(IF((Meilensteine[Status]&lt;&gt;"erledigt")*(Meilensteine[Plantermin]&gt;=TODAY()),Meilensteine[Plantermin]),2),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,Meilensteine!$C$2:$C$17/((Meilensteine!$E$2:$E$17&lt;&gt;"erledigt")*(Meilensteine!$C$2:$C$17&gt;=TODAY())),2),"")</f>
         <v/>
       </c>
       <c r="C19" s="4">
-        <f>IFERROR(INDEX(Meilensteine[Meilenstein],MATCH(B19,Meilensteine[Plantermin],0)),"")</f>
+        <f>IFERROR(INDEX(Meilensteine!$B$2:$B$17,MATCH(B19,Meilensteine!$C$2:$C$17,0)),"")</f>
         <v/>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="19">
-        <f>IFERROR(INDEX(Meilensteine[Status],MATCH(B19,Meilensteine[Plantermin],0)),"")</f>
+        <f>IFERROR(INDEX(Meilensteine!$E$2:$E$17,MATCH(B19,Meilensteine!$C$2:$C$17,0)),"")</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="18">
-        <f t="array" ref="B20">IFERROR(SMALL(IF((Meilensteine[Status]&lt;&gt;"erledigt")*(Meilensteine[Plantermin]&gt;=TODAY()),Meilensteine[Plantermin]),3),"")</f>
+        <f>IFERROR(AGGREGATE(15,6,Meilensteine!$C$2:$C$17/((Meilensteine!$E$2:$E$17&lt;&gt;"erledigt")*(Meilensteine!$C$2:$C$17&gt;=TODAY())),3),"")</f>
         <v/>
       </c>
       <c r="C20" s="4">
-        <f>IFERROR(INDEX(Meilensteine[Meilenstein],MATCH(B20,Meilensteine[Plantermin],0)),"")</f>
+        <f>IFERROR(INDEX(Meilensteine!$B$2:$B$17,MATCH(B20,Meilensteine!$C$2:$C$17,0)),"")</f>
         <v/>
       </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="19">
-        <f>IFERROR(INDEX(Meilensteine[Status],MATCH(B20,Meilensteine[Plantermin],0)),"")</f>
+        <f>IFERROR(INDEX(Meilensteine!$E$2:$E$17,MATCH(B20,Meilensteine!$C$2:$C$17,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C17">
     <cfRule type="expression" priority="5" dxfId="3">
-      <formula>AND($C2&lt;HEUTE();$E2&lt;&gt;"erledigt";$C2&lt;&gt;"")</formula>
+      <formula>AND($C2&lt;TODAY(),$E2&lt;&gt;"erledigt",$C2&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -2491,7 +2491,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E22">
     <cfRule type="expression" priority="6" dxfId="1">
-      <formula>AND($E2&lt;HEUTE();$F2&lt;&gt;"erledigt";$E2&lt;&gt;"")</formula>
+      <formula>AND($E2&lt;TODAY(),$F2&lt;&gt;"erledigt",$E2&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">

</xml_diff>

<commit_message>
Ausbau II: Lieferungen & Logistik, Testprotokolle, Budget & Fakturierung
Drei neue Blaetter (jetzt 12 gesamt):
- Lieferungen & Logistik: Anlieferungen, Kran/Lift, Tank mit 110%-Containment,
  Ruecktransporte, Demontage - mit Dropdowns und Status-Ampel
- Testprotokolle: Loadbank- und Heat-Load-Lastschritte (Soll/Ist), Ergebnis
  und Foto-Nachweis als Basis fuers Closeout-Paket
- Budget & Fakturierung: EUR-Einkaufsreferenzen (P-640380-3/P-650395-2) und
  Staffelungs-Fakturierung - ausdruecklich ohne CHF-Preise

Dashboard erweitert um KPIs 'Tests bestanden' und 'Lieferungen offen'.

Validierung: XML wohlgeformt, keine deutschen Funktionsnamen/Semikolons,
alle Tabellenspalten eindeutig, kein scharfes S, Strict-Reload ohne Warnungen.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YMxj9pzhuMuXneYjMXFmRT
</commit_message>
<xml_diff>
--- a/Projektsteuerung_MiT-PWR-WIN-2026-001.xlsx
+++ b/Projektsteuerung_MiT-PWR-WIN-2026-001.xlsx
@@ -12,10 +12,13 @@
     <sheet name="Meilensteine" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Aufgaben" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Personal &amp; Zutritt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Offene Punkte &amp; Risiken" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Dokumente" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Kontakte" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Aenderungslog" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Lieferungen &amp; Logistik" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Testprotokolle" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Offene Punkte &amp; Risiken" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Budget &amp; Fakturierung" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Dokumente" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Kontakte" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Aenderungslog" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Dashboard'!$A$1:$H$30</definedName>
@@ -24,10 +27,13 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Meilensteine'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Aufgaben'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Personal &amp; Zutritt'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Offene Punkte &amp; Risiken'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Dokumente'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Kontakte'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Aenderungslog'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Lieferungen &amp; Logistik'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Testprotokolle'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Offene Punkte &amp; Risiken'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Budget &amp; Fakturierung'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="9">'Dokumente'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="10">'Kontakte'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="11">'Aenderungslog'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -35,12 +41,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0&quot; Tage&quot;;&quot;ueberfaellig&quot;;&quot;heute&quot;"/>
     <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="167" formatCode="MMM"/>
     <numFmt numFmtId="168" formatCode="DD.MM.YYYY hh:mm"/>
+    <numFmt numFmtId="169" formatCode="#'##0&quot; EUR&quot;"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -212,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -283,6 +290,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -489,6 +499,18 @@
 </table>
 </file>
 
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Aenderungslog" displayName="Aenderungslog" ref="A1:C24" headerRowCount="1">
+  <autoFilter ref="A1:C24"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Datum"/>
+    <tableColumn id="2" name="Wer"/>
+    <tableColumn id="3" name="Was geaendert"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Aufgaben" displayName="Aufgaben" ref="A1:I22" headerRowCount="1">
   <autoFilter ref="A1:I22"/>
@@ -526,7 +548,45 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Risiken" displayName="Risiken" ref="A1:H10" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Logistik" displayName="Logistik" ref="A1:J8" headerRowCount="1">
+  <autoFilter ref="A1:J8"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="Nr."/>
+    <tableColumn id="2" name="Lieferung / Gegenstand"/>
+    <tableColumn id="3" name="Paket"/>
+    <tableColumn id="4" name="Anlieferung geplant"/>
+    <tableColumn id="5" name="Ort"/>
+    <tableColumn id="6" name="Kran/Lift"/>
+    <tableColumn id="7" name="Tank/Containment"/>
+    <tableColumn id="8" name="Verantwortlich"/>
+    <tableColumn id="9" name="Status"/>
+    <tableColumn id="10" name="Bemerkung"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Testprotokolle" displayName="Testprotokolle" ref="A1:J15" headerRowCount="1">
+  <autoFilter ref="A1:J15"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="Nr."/>
+    <tableColumn id="2" name="Test / Messung"/>
+    <tableColumn id="3" name="Paket"/>
+    <tableColumn id="4" name="Datum"/>
+    <tableColumn id="5" name="Sollwert"/>
+    <tableColumn id="6" name="Istwert"/>
+    <tableColumn id="7" name="Einheit"/>
+    <tableColumn id="8" name="Ergebnis"/>
+    <tableColumn id="9" name="Foto/Nachweis"/>
+    <tableColumn id="10" name="Bemerkung"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Risiken" displayName="Risiken" ref="A1:H10" headerRowCount="1">
   <autoFilter ref="A1:H10"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Nr."/>
@@ -542,8 +602,27 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Dokumente" displayName="Dokumente" ref="A1:F23" headerRowCount="1">
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Budget" displayName="Budget" ref="A1:J8" headerRowCount="1">
+  <autoFilter ref="A1:J8"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="Nr."/>
+    <tableColumn id="2" name="Kategorie"/>
+    <tableColumn id="3" name="Position"/>
+    <tableColumn id="4" name="Bezug (Angebot/PO)"/>
+    <tableColumn id="5" name="Paket"/>
+    <tableColumn id="6" name="Menge / Tage"/>
+    <tableColumn id="7" name="EUR (Referenz)"/>
+    <tableColumn id="8" name="Termin / Faelligkeit"/>
+    <tableColumn id="9" name="Status"/>
+    <tableColumn id="10" name="Bemerkung"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Dokumente" displayName="Dokumente" ref="A1:F23" headerRowCount="1">
   <autoFilter ref="A1:F23"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Nr."/>
@@ -557,8 +636,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Kontakte" displayName="Kontakte" ref="A1:H7" headerRowCount="1">
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Kontakte" displayName="Kontakte" ref="A1:H7" headerRowCount="1">
   <autoFilter ref="A1:H7"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Nr."/>
@@ -569,18 +648,6 @@
     <tableColumn id="6" name="E-Mail"/>
     <tableColumn id="7" name="Verfuegbarkeit"/>
     <tableColumn id="8" name="Bemerkung"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Aenderungslog" displayName="Aenderungslog" ref="A1:C23" headerRowCount="1">
-  <autoFilter ref="A1:C23"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Datum"/>
-    <tableColumn id="2" name="Wer"/>
-    <tableColumn id="3" name="Was geaendert"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -1208,6 +1275,11 @@
         <v/>
       </c>
       <c r="D20" s="5" t="n"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>TESTS &amp; LIEFERUNGEN</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="14" t="inlineStr">
@@ -1220,6 +1292,26 @@
         <v/>
       </c>
       <c r="D21" s="5" t="n"/>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>Tests bestanden</t>
+        </is>
+      </c>
+      <c r="F21" s="16">
+        <f>COUNTIF(Testprotokolle[Ergebnis],"bestanden")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>Lieferungen offen</t>
+        </is>
+      </c>
+      <c r="F22" s="16">
+        <f>COUNTIF(Logistik[Status],"offen")</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
@@ -1356,6 +1448,1170 @@
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Nr.</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>Dokument</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>Version/Datum</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>Quelle</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>Ablageort SharePoint</t>
+        </is>
+      </c>
+      <c r="F1" s="20" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>Angebot Aggreko P-640380-3 (Loadbank 6 MVA)</t>
+        </is>
+      </c>
+      <c r="C2" s="23" t="inlineStr"/>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>Aggreko</t>
+        </is>
+      </c>
+      <c r="E2" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F2" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="26" t="inlineStr">
+        <is>
+          <t>Angebot Aggreko P-650395-2 (Headload 8 MW)</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr"/>
+      <c r="D3" s="23" t="inlineStr">
+        <is>
+          <t>Aggreko</t>
+        </is>
+      </c>
+      <c r="E3" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F3" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>Purchase Order 49A (Loadbank)</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="inlineStr"/>
+      <c r="D4" s="23" t="inlineStr">
+        <is>
+          <t>DPR</t>
+        </is>
+      </c>
+      <c r="E4" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F4" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>Purchase Order 49B (Headload)</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr"/>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>DPR</t>
+        </is>
+      </c>
+      <c r="E5" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>NDA MiT-DPR</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr"/>
+      <c r="D6" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E6" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F6" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>Versicherungsnachweis</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr"/>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E7" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Logistikplan</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr"/>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Supplemental Conditions</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr"/>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>DPR</t>
+        </is>
+      </c>
+      <c r="E9" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Compliance-Unterlagen</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr"/>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>DPR</t>
+        </is>
+      </c>
+      <c r="E10" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>EHS-Plan Rev. 4</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Rev. 4</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>DPR</t>
+        </is>
+      </c>
+      <c r="E11" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Einzelanalyse 01</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr"/>
+      <c r="D12" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E12" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F12" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>Einzelanalyse 02</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr"/>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E13" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Einzelanalyse 03</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr"/>
+      <c r="D14" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E14" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>Einzelanalyse 04</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr"/>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E15" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Einzelanalyse 05</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr"/>
+      <c r="D16" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E16" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F16" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>Einzelanalyse 06</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr"/>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E17" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>Einzelanalyse 07</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr"/>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E18" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>Einzelanalyse 08</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr"/>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E19" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F19" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Einzelanalyse 09</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr"/>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E20" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F20" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>Einzelanalyse 10</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr"/>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E21" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Einzelanalyse 11</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr"/>
+      <c r="D22" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E22" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F22" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>Projektdossier (Gesamtuebersicht)</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="inlineStr"/>
+      <c r="D23" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E23" s="29" t="inlineStr">
+        <is>
+          <t>[SharePoint-Projektordner]</t>
+        </is>
+      </c>
+      <c r="F23" s="23" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="F2:F23">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
+      <formula>"signiert"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="5">
+      <formula>"final"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="9">
+      <formula>"ueberholt"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="D2:D23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"DPR,Aggreko,MiT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"Entwurf,final,signiert,ueberholt"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Nr.</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>Funktion</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>Firma</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>Telefon</t>
+        </is>
+      </c>
+      <c r="F1" s="20" t="inlineStr">
+        <is>
+          <t>E-Mail</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>Verfuegbarkeit</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>Bemerkung</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>Projektleiter MiT</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>Burak Uecoez</t>
+        </is>
+      </c>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E2" s="26" t="inlineStr">
+        <is>
+          <t>[eintragen]</t>
+        </is>
+      </c>
+      <c r="F2" s="26" t="inlineStr">
+        <is>
+          <t>[eintragen]</t>
+        </is>
+      </c>
+      <c r="G2" s="23" t="inlineStr">
+        <is>
+          <t>Buerozeiten</t>
+        </is>
+      </c>
+      <c r="H2" s="26" t="inlineStr">
+        <is>
+          <t>Gesamtverantwortung</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="26" t="inlineStr">
+        <is>
+          <t>DPR Bauleitung / Site Contact</t>
+        </is>
+      </c>
+      <c r="C3" s="26" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="D3" s="23" t="inlineStr">
+        <is>
+          <t>DPR</t>
+        </is>
+      </c>
+      <c r="E3" s="26" t="inlineStr">
+        <is>
+          <t>[eintragen]</t>
+        </is>
+      </c>
+      <c r="F3" s="26" t="inlineStr">
+        <is>
+          <t>[eintragen]</t>
+        </is>
+      </c>
+      <c r="G3" s="23" t="inlineStr">
+        <is>
+          <t>Buerozeiten</t>
+        </is>
+      </c>
+      <c r="H3" s="26" t="inlineStr">
+        <is>
+          <t>Hauptauftraggeber</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>Projektleiter Aggreko DE</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="D4" s="23" t="inlineStr">
+        <is>
+          <t>Aggreko</t>
+        </is>
+      </c>
+      <c r="E4" s="26" t="inlineStr">
+        <is>
+          <t>[eintragen]</t>
+        </is>
+      </c>
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>[eintragen]</t>
+        </is>
+      </c>
+      <c r="G4" s="23" t="inlineStr">
+        <is>
+          <t>Buerozeiten</t>
+        </is>
+      </c>
+      <c r="H4" s="26" t="inlineStr">
+        <is>
+          <t>Benennung ausstehend</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>Aggreko Service-Hotline</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>Aggreko</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>[eintragen]</t>
+        </is>
+      </c>
+      <c r="F5" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" s="23" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+      <c r="H5" s="26" t="inlineStr">
+        <is>
+          <t>Technische Stoerungen</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>MiT Notfall / Bereitschaft</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="inlineStr">
+        <is>
+          <t>MiT</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>[eintragen]</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" s="23" t="inlineStr">
+        <is>
+          <t>Bereitschaft</t>
+        </is>
+      </c>
+      <c r="H6" s="26" t="inlineStr">
+        <is>
+          <t>24/7-Kontaktkette</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>EHS / Sicherheit DPR</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>N.N.</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>DPR</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>[eintragen]</t>
+        </is>
+      </c>
+      <c r="F7" s="26" t="inlineStr">
+        <is>
+          <t>[eintragen]</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="inlineStr">
+        <is>
+          <t>Buerozeiten</t>
+        </is>
+      </c>
+      <c r="H7" s="26" t="inlineStr">
+        <is>
+          <t>EHS-Plan Rev. 4</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="G2:G7">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="10">
+      <formula>"24/7"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="D2:D7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"Aggreko,MiT,DPR"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"24/7,Buerozeiten,Bereitschaft"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>Wer</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>Was geaendert</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="22" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>Burak Uecoez</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>Projektsteuerungs-Tool erstellt und mit Projektdaten vorbefuellt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="22" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B3" s="26" t="inlineStr">
+        <is>
+          <t>Burak Uecoez</t>
+        </is>
+      </c>
+      <c r="C3" s="26" t="inlineStr">
+        <is>
+          <t>Erweiterung: Terminplan (Gantt), Personal &amp; Zutritt, Kontakte, Dashboard-Kennzahlen (Fortschritt, Countdowns, Ampel).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="22" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>Burak Uecoez</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>Ergaenzt: Lieferungen &amp; Logistik, Testprotokolle (Testnachweise fuer Closeout), Budget &amp; Fakturierung (nur EUR-Referenz).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="22" t="n"/>
+      <c r="B5" s="26" t="n"/>
+      <c r="C5" s="26" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="22" t="n"/>
+      <c r="B6" s="26" t="n"/>
+      <c r="C6" s="26" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="n"/>
+      <c r="B7" s="26" t="n"/>
+      <c r="C7" s="26" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="n"/>
+      <c r="B8" s="26" t="n"/>
+      <c r="C8" s="26" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="n"/>
+      <c r="B9" s="26" t="n"/>
+      <c r="C9" s="26" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="n"/>
+      <c r="B10" s="26" t="n"/>
+      <c r="C10" s="26" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="n"/>
+      <c r="B11" s="26" t="n"/>
+      <c r="C11" s="26" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="22" t="n"/>
+      <c r="B12" s="26" t="n"/>
+      <c r="C12" s="26" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="n"/>
+      <c r="B13" s="26" t="n"/>
+      <c r="C13" s="26" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="n"/>
+      <c r="B14" s="26" t="n"/>
+      <c r="C14" s="26" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="n"/>
+      <c r="B15" s="26" t="n"/>
+      <c r="C15" s="26" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="n"/>
+      <c r="B16" s="26" t="n"/>
+      <c r="C16" s="26" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="n"/>
+      <c r="B17" s="26" t="n"/>
+      <c r="C17" s="26" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="22" t="n"/>
+      <c r="B18" s="26" t="n"/>
+      <c r="C18" s="26" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="n"/>
+      <c r="B19" s="26" t="n"/>
+      <c r="C19" s="26" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="n"/>
+      <c r="B20" s="26" t="n"/>
+      <c r="C20" s="26" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="n"/>
+      <c r="B21" s="26" t="n"/>
+      <c r="C21" s="26" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="n"/>
+      <c r="B22" s="26" t="n"/>
+      <c r="C22" s="26" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="22" t="n"/>
+      <c r="B23" s="26" t="n"/>
+      <c r="C23" s="26" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="n"/>
+      <c r="B24" s="26" t="n"/>
+      <c r="C24" s="26" t="n"/>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3411,6 +4667,1076 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Nr.</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>Lieferung / Gegenstand</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>Paket</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>Anlieferung geplant</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>Ort</t>
+        </is>
+      </c>
+      <c r="F1" s="20" t="inlineStr">
+        <is>
+          <t>Kran/Lift</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>Tank/Containment</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>Verantwortlich</t>
+        </is>
+      </c>
+      <c r="I1" s="20" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="20" t="inlineStr">
+        <is>
+          <t>Bemerkung</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>Headloads (54x 200 kW)</t>
+        </is>
+      </c>
+      <c r="C2" s="23" t="inlineStr">
+        <is>
+          <t>Headload</t>
+        </is>
+      </c>
+      <c r="D2" s="22" t="n">
+        <v>46237</v>
+      </c>
+      <c r="E2" s="26" t="inlineStr">
+        <is>
+          <t>ZRH12 Winterthur</t>
+        </is>
+      </c>
+      <c r="F2" s="23" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G2" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2" s="23" t="inlineStr">
+        <is>
+          <t>Aggreko</t>
+        </is>
+      </c>
+      <c r="I2" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J2" s="26" t="inlineStr">
+        <is>
+          <t>Lift Plan erforderlich</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="26" t="inlineStr">
+        <is>
+          <t>Loadbank 6 MVA</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>Loadbank</t>
+        </is>
+      </c>
+      <c r="D3" s="22" t="n">
+        <v>46251</v>
+      </c>
+      <c r="E3" s="26" t="inlineStr">
+        <is>
+          <t>ZRH12 Winterthur</t>
+        </is>
+      </c>
+      <c r="F3" s="23" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G3" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H3" s="23" t="inlineStr">
+        <is>
+          <t>Aggreko</t>
+        </is>
+      </c>
+      <c r="I3" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J3" s="26" t="inlineStr">
+        <is>
+          <t>Kranfrage klaeren</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>Tank / Betankung</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
+          <t>Headload</t>
+        </is>
+      </c>
+      <c r="D4" s="23" t="inlineStr">
+        <is>
+          <t>vor Testbeginn</t>
+        </is>
+      </c>
+      <c r="E4" s="26" t="inlineStr">
+        <is>
+          <t>ZRH12 Winterthur</t>
+        </is>
+      </c>
+      <c r="F4" s="23" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="G4" s="26" t="inlineStr">
+        <is>
+          <t>110%-Containment</t>
+        </is>
+      </c>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>Burak</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J4" s="26" t="inlineStr">
+        <is>
+          <t>Standort festlegen</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>Kabel- &amp; Anschlussmaterial</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>vor Testbeginn</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>ZRH12 Winterthur</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="G5" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>Aggreko</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J5" s="26" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>Ruecktransport Loadbank</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>Loadbank</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="n">
+        <v>46328</v>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>ab ZRH12</t>
+        </is>
+      </c>
+      <c r="F6" s="23" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G6" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>Aggreko</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J6" s="26" t="inlineStr">
+        <is>
+          <t>nach Mietende</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>Ruecktransport Headloads</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>Headload</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>46367</v>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>ab ZRH12</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G7" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>Aggreko</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J7" s="26" t="inlineStr">
+        <is>
+          <t>nach Mietende</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Demontage &amp; Abtransport</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>46370</v>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>ZRH12 Winterthur</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G8" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>Aggreko</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J8" s="26" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="I2:I8">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
+      <formula>"geliefert"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
+      <formula>"zurueck"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="6">
+      <formula>"verschoben"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="5">
+      <formula>"geplant"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="4">
+    <dataValidation sqref="C2:C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"Loadbank,Headload,beide"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"ja,nein,offen"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"Burak,Aggreko,DPR,MiT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"offen,geplant,geliefert,zurueck,verschoben"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Nr.</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>Test / Messung</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>Paket</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>Sollwert</t>
+        </is>
+      </c>
+      <c r="F1" s="20" t="inlineStr">
+        <is>
+          <t>Istwert</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>Einheit</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>Ergebnis</t>
+        </is>
+      </c>
+      <c r="I1" s="20" t="inlineStr">
+        <is>
+          <t>Foto/Nachweis</t>
+        </is>
+      </c>
+      <c r="J1" s="20" t="inlineStr">
+        <is>
+          <t>Bemerkung</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>Sichtpruefung &amp; Anschlusskontrolle</t>
+        </is>
+      </c>
+      <c r="C2" s="23" t="inlineStr">
+        <is>
+          <t>Loadbank</t>
+        </is>
+      </c>
+      <c r="D2" s="22" t="n"/>
+      <c r="E2" s="23" t="inlineStr">
+        <is>
+          <t>i.O.</t>
+        </is>
+      </c>
+      <c r="F2" s="23" t="n"/>
+      <c r="G2" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I2" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J2" s="26" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="26" t="inlineStr">
+        <is>
+          <t>Isolationspruefung</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>Loadbank</t>
+        </is>
+      </c>
+      <c r="D3" s="22" t="n"/>
+      <c r="E3" s="23" t="inlineStr"/>
+      <c r="F3" s="23" t="n"/>
+      <c r="G3" s="23" t="inlineStr">
+        <is>
+          <t>MOhm</t>
+        </is>
+      </c>
+      <c r="H3" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I3" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J3" s="26" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>Lastschritt 25% (1.5 MVA)</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
+          <t>Loadbank</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="n"/>
+      <c r="E4" s="23" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F4" s="23" t="n"/>
+      <c r="G4" s="23" t="inlineStr">
+        <is>
+          <t>MVA</t>
+        </is>
+      </c>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J4" s="26" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>Lastschritt 50% (3.0 MVA)</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>Loadbank</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="23" t="n"/>
+      <c r="G5" s="23" t="inlineStr">
+        <is>
+          <t>MVA</t>
+        </is>
+      </c>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J5" s="26" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>Lastschritt 75% (4.5 MVA)</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>Loadbank</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="23" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F6" s="23" t="n"/>
+      <c r="G6" s="23" t="inlineStr">
+        <is>
+          <t>MVA</t>
+        </is>
+      </c>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J6" s="26" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>Lastschritt 100% (6.0 MVA)</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>Loadbank</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="n"/>
+      <c r="E7" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" s="23" t="n"/>
+      <c r="G7" s="23" t="inlineStr">
+        <is>
+          <t>MVA</t>
+        </is>
+      </c>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J7" s="26" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Frequenzstabilitaet</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Loadbank</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="n"/>
+      <c r="E8" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="F8" s="23" t="n"/>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>Hz</t>
+        </is>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J8" s="26" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Sichtpruefung Headloads</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>Headload</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>i.O.</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="n"/>
+      <c r="G9" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J9" s="26" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Lastschritt 2 MW</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>Headload</t>
+        </is>
+      </c>
+      <c r="D10" s="22" t="n"/>
+      <c r="E10" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="23" t="n"/>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J10" s="26" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Lastschritt 4 MW</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Headload</t>
+        </is>
+      </c>
+      <c r="D11" s="22" t="n"/>
+      <c r="E11" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" s="23" t="n"/>
+      <c r="G11" s="23" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J11" s="26" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Lastschritt 6 MW</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>Headload</t>
+        </is>
+      </c>
+      <c r="D12" s="22" t="n"/>
+      <c r="E12" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="F12" s="23" t="n"/>
+      <c r="G12" s="23" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J12" s="26" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>Lastschritt 8 MW (Volllast)</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>Headload</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="n"/>
+      <c r="E13" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" s="23" t="n"/>
+      <c r="G13" s="23" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I13" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J13" s="26" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Waermeabfuhr-Nachweis (Dauerlauf)</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>Headload</t>
+        </is>
+      </c>
+      <c r="D14" s="22" t="n"/>
+      <c r="E14" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="n"/>
+      <c r="G14" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J14" s="26" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>Not-Aus / Sicherheitskette</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="n"/>
+      <c r="E15" s="23" t="inlineStr">
+        <is>
+          <t>i.O.</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="n"/>
+      <c r="G15" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J15" s="26" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>Istwerte, Datum und Foto-Nachweis vor Ort eintragen. Ergebnis = Basis fuer das Closeout-Paket.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B17:J17"/>
+  </mergeCells>
+  <conditionalFormatting sqref="H2:H15">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
+      <formula>"bestanden"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
+      <formula>"nicht bestanden"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I15">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3">
+      <formula>"ja"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation sqref="C2:C15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"Loadbank,Headload,beide"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"bestanden,nicht bestanden,offen,n.a."</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"ja,nein,offen"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3848,21 +6174,25 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3873,27 +6203,47 @@
       </c>
       <c r="B1" s="20" t="inlineStr">
         <is>
-          <t>Dokument</t>
+          <t>Kategorie</t>
         </is>
       </c>
       <c r="C1" s="20" t="inlineStr">
         <is>
-          <t>Version/Datum</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D1" s="20" t="inlineStr">
         <is>
-          <t>Quelle</t>
+          <t>Bezug (Angebot/PO)</t>
         </is>
       </c>
       <c r="E1" s="20" t="inlineStr">
         <is>
-          <t>Ablageort SharePoint</t>
+          <t>Paket</t>
         </is>
       </c>
       <c r="F1" s="20" t="inlineStr">
         <is>
+          <t>Menge / Tage</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>EUR (Referenz)</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>Termin / Faelligkeit</t>
+        </is>
+      </c>
+      <c r="I1" s="20" t="inlineStr">
+        <is>
           <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="20" t="inlineStr">
+        <is>
+          <t>Bemerkung</t>
         </is>
       </c>
     </row>
@@ -3901,25 +6251,43 @@
       <c r="A2" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="26" t="inlineStr">
-        <is>
-          <t>Angebot Aggreko P-640380-3 (Loadbank 6 MVA)</t>
-        </is>
-      </c>
-      <c r="C2" s="23" t="inlineStr"/>
-      <c r="D2" s="23" t="inlineStr">
-        <is>
-          <t>Aggreko</t>
-        </is>
-      </c>
-      <c r="E2" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F2" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>Einkauf-Referenz</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>Loadbank 6 MVA - Miete</t>
+        </is>
+      </c>
+      <c r="D2" s="26" t="inlineStr">
+        <is>
+          <t>P-640380-3</t>
+        </is>
+      </c>
+      <c r="E2" s="23" t="inlineStr">
+        <is>
+          <t>Loadbank</t>
+        </is>
+      </c>
+      <c r="F2" s="23" t="n">
+        <v>110</v>
+      </c>
+      <c r="G2" s="28" t="n"/>
+      <c r="H2" s="26" t="inlineStr">
+        <is>
+          <t>Mietende 02.11.</t>
+        </is>
+      </c>
+      <c r="I2" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J2" s="26" t="inlineStr">
+        <is>
+          <t>Basis 110 Tage; PO-Pruefung 78/131 falsch</t>
         </is>
       </c>
     </row>
@@ -3927,51 +6295,81 @@
       <c r="A3" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="26" t="inlineStr">
-        <is>
-          <t>Angebot Aggreko P-650395-2 (Headload 8 MW)</t>
-        </is>
-      </c>
-      <c r="C3" s="23" t="inlineStr"/>
-      <c r="D3" s="23" t="inlineStr">
-        <is>
-          <t>Aggreko</t>
-        </is>
-      </c>
-      <c r="E3" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F3" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Einkauf-Referenz</t>
+        </is>
+      </c>
+      <c r="C3" s="26" t="inlineStr">
+        <is>
+          <t>Headload 8 MW - Miete</t>
+        </is>
+      </c>
+      <c r="D3" s="26" t="inlineStr">
+        <is>
+          <t>P-650395-2</t>
+        </is>
+      </c>
+      <c r="E3" s="23" t="inlineStr">
+        <is>
+          <t>Headload</t>
+        </is>
+      </c>
+      <c r="F3" s="23" t="n">
+        <v>110</v>
+      </c>
+      <c r="G3" s="28" t="n"/>
+      <c r="H3" s="26" t="inlineStr">
+        <is>
+          <t>Mietende 11.12.</t>
+        </is>
+      </c>
+      <c r="I3" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J3" s="26" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="26" t="inlineStr">
-        <is>
-          <t>Purchase Order 49A (Loadbank)</t>
-        </is>
-      </c>
-      <c r="C4" s="23" t="inlineStr"/>
-      <c r="D4" s="23" t="inlineStr">
-        <is>
-          <t>DPR</t>
-        </is>
-      </c>
-      <c r="E4" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F4" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>Logistik</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>Transport / Kran / Lift</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" s="23" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="F4" s="23" t="n"/>
+      <c r="G4" s="28" t="n"/>
+      <c r="H4" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J4" s="26" t="inlineStr">
+        <is>
+          <t>Details in Lieferungen &amp; Logistik</t>
         </is>
       </c>
     </row>
@@ -3979,25 +6377,41 @@
       <c r="A5" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="26" t="inlineStr">
-        <is>
-          <t>Purchase Order 49B (Headload)</t>
-        </is>
-      </c>
-      <c r="C5" s="23" t="inlineStr"/>
-      <c r="D5" s="23" t="inlineStr">
-        <is>
-          <t>DPR</t>
-        </is>
-      </c>
-      <c r="E5" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F5" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>Kraftstoff</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>Betankung (separat)</t>
+        </is>
+      </c>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>Headload</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="n"/>
+      <c r="G5" s="28" t="n"/>
+      <c r="H5" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J5" s="26" t="inlineStr">
+        <is>
+          <t>Zollprozess: Kraftstoff vs. Equipment</t>
         </is>
       </c>
     </row>
@@ -4005,25 +6419,41 @@
       <c r="A6" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="26" t="inlineStr">
-        <is>
-          <t>NDA MiT-DPR</t>
-        </is>
-      </c>
-      <c r="C6" s="23" t="inlineStr"/>
-      <c r="D6" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E6" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F6" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>Fakturierung</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>Rate 1 (Staffelung)</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>PO 49A/49B</t>
+        </is>
+      </c>
+      <c r="E6" s="23" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="F6" s="23" t="n"/>
+      <c r="G6" s="28" t="n"/>
+      <c r="H6" s="26" t="inlineStr">
+        <is>
+          <t>n. Abstimmung</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J6" s="26" t="inlineStr">
+        <is>
+          <t>Staffelungs-Fakturierung klaeren</t>
         </is>
       </c>
     </row>
@@ -4031,466 +6461,113 @@
       <c r="A7" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="26" t="inlineStr">
-        <is>
-          <t>Versicherungsnachweis</t>
-        </is>
-      </c>
-      <c r="C7" s="23" t="inlineStr"/>
-      <c r="D7" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E7" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F7" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>Fakturierung</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>Rate 2 (Staffelung)</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>PO 49A/49B</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="n"/>
+      <c r="G7" s="28" t="n"/>
+      <c r="H7" s="26" t="inlineStr">
+        <is>
+          <t>n. Abstimmung</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J7" s="26" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="23" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="26" t="inlineStr">
-        <is>
-          <t>Logistikplan</t>
-        </is>
-      </c>
-      <c r="C8" s="23" t="inlineStr"/>
-      <c r="D8" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E8" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F8" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="26" t="inlineStr">
-        <is>
-          <t>Supplemental Conditions</t>
-        </is>
-      </c>
-      <c r="C9" s="23" t="inlineStr"/>
-      <c r="D9" s="23" t="inlineStr">
-        <is>
-          <t>DPR</t>
-        </is>
-      </c>
-      <c r="E9" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F9" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Fakturierung</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>Schlussrechnung</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>PO 49A/49B</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="n"/>
+      <c r="G8" s="28" t="n"/>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>Closeout Dez.</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="J8" s="26" t="inlineStr">
+        <is>
+          <t>nach Abnahme</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="26" t="inlineStr">
-        <is>
-          <t>Compliance-Unterlagen</t>
-        </is>
-      </c>
-      <c r="C10" s="23" t="inlineStr"/>
-      <c r="D10" s="23" t="inlineStr">
-        <is>
-          <t>DPR</t>
-        </is>
-      </c>
-      <c r="E10" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F10" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="26" t="inlineStr">
-        <is>
-          <t>EHS-Plan Rev. 4</t>
-        </is>
-      </c>
-      <c r="C11" s="23" t="inlineStr">
-        <is>
-          <t>Rev. 4</t>
-        </is>
-      </c>
-      <c r="D11" s="23" t="inlineStr">
-        <is>
-          <t>DPR</t>
-        </is>
-      </c>
-      <c r="E11" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F11" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="23" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="26" t="inlineStr">
-        <is>
-          <t>Einzelanalyse 01</t>
-        </is>
-      </c>
-      <c r="C12" s="23" t="inlineStr"/>
-      <c r="D12" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E12" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F12" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="23" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="26" t="inlineStr">
-        <is>
-          <t>Einzelanalyse 02</t>
-        </is>
-      </c>
-      <c r="C13" s="23" t="inlineStr"/>
-      <c r="D13" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E13" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F13" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="23" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="26" t="inlineStr">
-        <is>
-          <t>Einzelanalyse 03</t>
-        </is>
-      </c>
-      <c r="C14" s="23" t="inlineStr"/>
-      <c r="D14" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E14" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F14" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="23" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="26" t="inlineStr">
-        <is>
-          <t>Einzelanalyse 04</t>
-        </is>
-      </c>
-      <c r="C15" s="23" t="inlineStr"/>
-      <c r="D15" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E15" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F15" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="23" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="26" t="inlineStr">
-        <is>
-          <t>Einzelanalyse 05</t>
-        </is>
-      </c>
-      <c r="C16" s="23" t="inlineStr"/>
-      <c r="D16" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E16" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F16" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="23" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="26" t="inlineStr">
-        <is>
-          <t>Einzelanalyse 06</t>
-        </is>
-      </c>
-      <c r="C17" s="23" t="inlineStr"/>
-      <c r="D17" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E17" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F17" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="23" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="26" t="inlineStr">
-        <is>
-          <t>Einzelanalyse 07</t>
-        </is>
-      </c>
-      <c r="C18" s="23" t="inlineStr"/>
-      <c r="D18" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E18" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F18" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="23" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="26" t="inlineStr">
-        <is>
-          <t>Einzelanalyse 08</t>
-        </is>
-      </c>
-      <c r="C19" s="23" t="inlineStr"/>
-      <c r="D19" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E19" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F19" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="23" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="26" t="inlineStr">
-        <is>
-          <t>Einzelanalyse 09</t>
-        </is>
-      </c>
-      <c r="C20" s="23" t="inlineStr"/>
-      <c r="D20" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E20" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F20" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="23" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="26" t="inlineStr">
-        <is>
-          <t>Einzelanalyse 10</t>
-        </is>
-      </c>
-      <c r="C21" s="23" t="inlineStr"/>
-      <c r="D21" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E21" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F21" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="23" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="26" t="inlineStr">
-        <is>
-          <t>Einzelanalyse 11</t>
-        </is>
-      </c>
-      <c r="C22" s="23" t="inlineStr"/>
-      <c r="D22" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E22" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F22" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="23" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="26" t="inlineStr">
-        <is>
-          <t>Projektdossier (Gesamtuebersicht)</t>
-        </is>
-      </c>
-      <c r="C23" s="23" t="inlineStr"/>
-      <c r="D23" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E23" s="28" t="inlineStr">
-        <is>
-          <t>[SharePoint-Projektordner]</t>
-        </is>
-      </c>
-      <c r="F23" s="23" t="inlineStr">
-        <is>
-          <t>Entwurf</t>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>Nur EUR-Einkaufsreferenzen aus den Aggreko-Angeboten. KEINE CHF-Preise (Vertraulichkeit / Marge).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F23">
+  <mergeCells count="1">
+    <mergeCell ref="B10:J10"/>
+  </mergeCells>
+  <conditionalFormatting sqref="I2:I8">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
-      <formula>"signiert"</formula>
+      <formula>"bezahlt"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="5">
-      <formula>"final"</formula>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
+      <formula>"geprueft"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="9">
-      <formula>"ueberholt"</formula>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
+      <formula>"gestellt"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation sqref="D2:D23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
-      <formula1>"DPR,Aggreko,MiT"</formula1>
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"Einkauf-Referenz,Fakturierung,Logistik,Kraftstoff"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
-      <formula1>"Entwurf,final,signiert,ueberholt"</formula1>
+    <dataValidation sqref="E2:E8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"Loadbank,Headload,beide"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+      <formula1>"offen,gestellt,bezahlt,geprueft"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
@@ -4500,499 +6577,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="20" t="inlineStr">
-        <is>
-          <t>Nr.</t>
-        </is>
-      </c>
-      <c r="B1" s="20" t="inlineStr">
-        <is>
-          <t>Funktion</t>
-        </is>
-      </c>
-      <c r="C1" s="20" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="D1" s="20" t="inlineStr">
-        <is>
-          <t>Firma</t>
-        </is>
-      </c>
-      <c r="E1" s="20" t="inlineStr">
-        <is>
-          <t>Telefon</t>
-        </is>
-      </c>
-      <c r="F1" s="20" t="inlineStr">
-        <is>
-          <t>E-Mail</t>
-        </is>
-      </c>
-      <c r="G1" s="20" t="inlineStr">
-        <is>
-          <t>Verfuegbarkeit</t>
-        </is>
-      </c>
-      <c r="H1" s="20" t="inlineStr">
-        <is>
-          <t>Bemerkung</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="26" t="inlineStr">
-        <is>
-          <t>Projektleiter MiT</t>
-        </is>
-      </c>
-      <c r="C2" s="26" t="inlineStr">
-        <is>
-          <t>Burak Uecoez</t>
-        </is>
-      </c>
-      <c r="D2" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E2" s="26" t="inlineStr">
-        <is>
-          <t>[eintragen]</t>
-        </is>
-      </c>
-      <c r="F2" s="26" t="inlineStr">
-        <is>
-          <t>[eintragen]</t>
-        </is>
-      </c>
-      <c r="G2" s="23" t="inlineStr">
-        <is>
-          <t>Buerozeiten</t>
-        </is>
-      </c>
-      <c r="H2" s="26" t="inlineStr">
-        <is>
-          <t>Gesamtverantwortung</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="26" t="inlineStr">
-        <is>
-          <t>DPR Bauleitung / Site Contact</t>
-        </is>
-      </c>
-      <c r="C3" s="26" t="inlineStr">
-        <is>
-          <t>N.N.</t>
-        </is>
-      </c>
-      <c r="D3" s="23" t="inlineStr">
-        <is>
-          <t>DPR</t>
-        </is>
-      </c>
-      <c r="E3" s="26" t="inlineStr">
-        <is>
-          <t>[eintragen]</t>
-        </is>
-      </c>
-      <c r="F3" s="26" t="inlineStr">
-        <is>
-          <t>[eintragen]</t>
-        </is>
-      </c>
-      <c r="G3" s="23" t="inlineStr">
-        <is>
-          <t>Buerozeiten</t>
-        </is>
-      </c>
-      <c r="H3" s="26" t="inlineStr">
-        <is>
-          <t>Hauptauftraggeber</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="26" t="inlineStr">
-        <is>
-          <t>Projektleiter Aggreko DE</t>
-        </is>
-      </c>
-      <c r="C4" s="26" t="inlineStr">
-        <is>
-          <t>N.N.</t>
-        </is>
-      </c>
-      <c r="D4" s="23" t="inlineStr">
-        <is>
-          <t>Aggreko</t>
-        </is>
-      </c>
-      <c r="E4" s="26" t="inlineStr">
-        <is>
-          <t>[eintragen]</t>
-        </is>
-      </c>
-      <c r="F4" s="26" t="inlineStr">
-        <is>
-          <t>[eintragen]</t>
-        </is>
-      </c>
-      <c r="G4" s="23" t="inlineStr">
-        <is>
-          <t>Buerozeiten</t>
-        </is>
-      </c>
-      <c r="H4" s="26" t="inlineStr">
-        <is>
-          <t>Benennung ausstehend</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="26" t="inlineStr">
-        <is>
-          <t>Aggreko Service-Hotline</t>
-        </is>
-      </c>
-      <c r="C5" s="26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D5" s="23" t="inlineStr">
-        <is>
-          <t>Aggreko</t>
-        </is>
-      </c>
-      <c r="E5" s="26" t="inlineStr">
-        <is>
-          <t>[eintragen]</t>
-        </is>
-      </c>
-      <c r="F5" s="26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G5" s="23" t="inlineStr">
-        <is>
-          <t>24/7</t>
-        </is>
-      </c>
-      <c r="H5" s="26" t="inlineStr">
-        <is>
-          <t>Technische Stoerungen</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="26" t="inlineStr">
-        <is>
-          <t>MiT Notfall / Bereitschaft</t>
-        </is>
-      </c>
-      <c r="C6" s="26" t="inlineStr">
-        <is>
-          <t>N.N.</t>
-        </is>
-      </c>
-      <c r="D6" s="23" t="inlineStr">
-        <is>
-          <t>MiT</t>
-        </is>
-      </c>
-      <c r="E6" s="26" t="inlineStr">
-        <is>
-          <t>[eintragen]</t>
-        </is>
-      </c>
-      <c r="F6" s="26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G6" s="23" t="inlineStr">
-        <is>
-          <t>Bereitschaft</t>
-        </is>
-      </c>
-      <c r="H6" s="26" t="inlineStr">
-        <is>
-          <t>24/7-Kontaktkette</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="26" t="inlineStr">
-        <is>
-          <t>EHS / Sicherheit DPR</t>
-        </is>
-      </c>
-      <c r="C7" s="26" t="inlineStr">
-        <is>
-          <t>N.N.</t>
-        </is>
-      </c>
-      <c r="D7" s="23" t="inlineStr">
-        <is>
-          <t>DPR</t>
-        </is>
-      </c>
-      <c r="E7" s="26" t="inlineStr">
-        <is>
-          <t>[eintragen]</t>
-        </is>
-      </c>
-      <c r="F7" s="26" t="inlineStr">
-        <is>
-          <t>[eintragen]</t>
-        </is>
-      </c>
-      <c r="G7" s="23" t="inlineStr">
-        <is>
-          <t>Buerozeiten</t>
-        </is>
-      </c>
-      <c r="H7" s="26" t="inlineStr">
-        <is>
-          <t>EHS-Plan Rev. 4</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="G2:G7">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="10">
-      <formula>"24/7"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation sqref="D2:D7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
-      <formula1>"Aggreko,MiT,DPR"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
-      <formula1>"24/7,Buerozeiten,Bereitschaft"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:C23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="20" t="inlineStr">
-        <is>
-          <t>Datum</t>
-        </is>
-      </c>
-      <c r="B1" s="20" t="inlineStr">
-        <is>
-          <t>Wer</t>
-        </is>
-      </c>
-      <c r="C1" s="20" t="inlineStr">
-        <is>
-          <t>Was geaendert</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="22" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B2" s="26" t="inlineStr">
-        <is>
-          <t>Burak Uecoez</t>
-        </is>
-      </c>
-      <c r="C2" s="26" t="inlineStr">
-        <is>
-          <t>Projektsteuerungs-Tool erstellt und mit Projektdaten vorbefuellt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="22" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B3" s="26" t="inlineStr">
-        <is>
-          <t>Burak Uecoez</t>
-        </is>
-      </c>
-      <c r="C3" s="26" t="inlineStr">
-        <is>
-          <t>Erweiterung: Terminplan (Gantt), Personal &amp; Zutritt, Kontakte, Dashboard-Kennzahlen (Fortschritt, Countdowns, Ampel).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="22" t="n"/>
-      <c r="B4" s="26" t="n"/>
-      <c r="C4" s="26" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="22" t="n"/>
-      <c r="B5" s="26" t="n"/>
-      <c r="C5" s="26" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="22" t="n"/>
-      <c r="B6" s="26" t="n"/>
-      <c r="C6" s="26" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="22" t="n"/>
-      <c r="B7" s="26" t="n"/>
-      <c r="C7" s="26" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="22" t="n"/>
-      <c r="B8" s="26" t="n"/>
-      <c r="C8" s="26" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="22" t="n"/>
-      <c r="B9" s="26" t="n"/>
-      <c r="C9" s="26" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="22" t="n"/>
-      <c r="B10" s="26" t="n"/>
-      <c r="C10" s="26" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="22" t="n"/>
-      <c r="B11" s="26" t="n"/>
-      <c r="C11" s="26" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="22" t="n"/>
-      <c r="B12" s="26" t="n"/>
-      <c r="C12" s="26" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="22" t="n"/>
-      <c r="B13" s="26" t="n"/>
-      <c r="C13" s="26" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="22" t="n"/>
-      <c r="B14" s="26" t="n"/>
-      <c r="C14" s="26" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="22" t="n"/>
-      <c r="B15" s="26" t="n"/>
-      <c r="C15" s="26" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="22" t="n"/>
-      <c r="B16" s="26" t="n"/>
-      <c r="C16" s="26" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="22" t="n"/>
-      <c r="B17" s="26" t="n"/>
-      <c r="C17" s="26" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="22" t="n"/>
-      <c r="B18" s="26" t="n"/>
-      <c r="C18" s="26" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="22" t="n"/>
-      <c r="B19" s="26" t="n"/>
-      <c r="C19" s="26" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="22" t="n"/>
-      <c r="B20" s="26" t="n"/>
-      <c r="C20" s="26" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="22" t="n"/>
-      <c r="B21" s="26" t="n"/>
-      <c r="C21" s="26" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="22" t="n"/>
-      <c r="B22" s="26" t="n"/>
-      <c r="C22" s="26" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="22" t="n"/>
-      <c r="B23" s="26" t="n"/>
-      <c r="C23" s="26" t="n"/>
-    </row>
-  </sheetData>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Kalender-Gegenpruefung 2026: 3 Samstag-Termine korrigiert
Vollstaendige Verifikation aller Termine gegen den ISO-Kalender 2026:
- Alle 25 Gantt-Wochenspalten sind echte Montage mit korrekter ISO-KW
  (KW29 = 13.-19.07.2026 bis KW53 = 28.12.2026), unabhaengig verifiziert
- Alle 24 Meilensteine liegen auf Werktagen mit korrekter KW

Korrigiert (fielen auf Samstage):
- NDA MiT-DPR anstossen: 18.07. -> 17.07. (Fr, vor Unterzeichnung 22.07.)
- WORKcontrol-Registrierung: 25.07. -> 24.07. (Fr, vor Badges 03.08.)
- 24/7-Kontaktkette: 01.08. (Sa + Bundesfeier CH) -> 31.07. (Fr)

Zudem: Balken-Chart nach H31 verschoben (keine Ueberlappung mit Doughnut),
Druckbereich Dashboard auf A1:M49 erweitert, Aenderungslog ergaenzt.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YMxj9pzhuMuXneYjMXFmRT
</commit_message>
<xml_diff>
--- a/Projektsteuerung_MiT-PWR-WIN-2026-001.xlsx
+++ b/Projektsteuerung_MiT-PWR-WIN-2026-001.xlsx
@@ -21,7 +21,7 @@
     <sheet name="Aenderungslog" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Dashboard'!$A$1:$H$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Dashboard'!$A$1:$M$49</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Terminplan'!$2:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Meilensteine'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Aufgaben'!$1:$1</definedName>
@@ -837,7 +837,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>7</col>
       <colOff>0</colOff>
       <row>30</row>
       <rowOff>0</rowOff>
@@ -880,8 +880,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Aenderungslog" displayName="Aenderungslog" ref="A1:C26" headerRowCount="1">
-  <autoFilter ref="A1:C26"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Aenderungslog" displayName="Aenderungslog" ref="A1:C27" headerRowCount="1">
+  <autoFilter ref="A1:C27"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Datum"/>
     <tableColumn id="2" name="Wer"/>
@@ -3040,7 +3040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3141,9 +3141,19 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="n"/>
-      <c r="B7" s="34" t="n"/>
-      <c r="C7" s="34" t="n"/>
+      <c r="A7" s="25" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B7" s="34" t="inlineStr">
+        <is>
+          <t>Burak Uecoez</t>
+        </is>
+      </c>
+      <c r="C7" s="34" t="inlineStr">
+        <is>
+          <t>Kalender-Gegenpruefung 2026: alle KW/Wochentage verifiziert; 3 Samstag-Termine korrigiert (NDA 17.07., WORKcontrol 24.07., Kontaktkette 31.07. statt 01.08./Bundesfeier).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="25" t="n"/>
@@ -3239,6 +3249,11 @@
       <c r="A26" s="25" t="n"/>
       <c r="B26" s="34" t="n"/>
       <c r="C26" s="34" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="25" t="n"/>
+      <c r="B27" s="34" t="n"/>
+      <c r="C27" s="34" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1"/>
@@ -8206,7 +8221,7 @@
         </is>
       </c>
       <c r="E7" s="25" t="n">
-        <v>46228</v>
+        <v>46227</v>
       </c>
       <c r="F7" s="30" t="inlineStr">
         <is>
@@ -8220,7 +8235,7 @@
       </c>
       <c r="H7" s="34" t="inlineStr">
         <is>
-          <t>vor Badges</t>
+          <t>vor Badges (25.07. = Samstag)</t>
         </is>
       </c>
       <c r="I7" s="25" t="n"/>
@@ -8650,7 +8665,7 @@
         </is>
       </c>
       <c r="E19" s="25" t="n">
-        <v>46221</v>
+        <v>46220</v>
       </c>
       <c r="F19" s="30" t="inlineStr">
         <is>
@@ -8664,7 +8679,7 @@
       </c>
       <c r="H19" s="34" t="inlineStr">
         <is>
-          <t>eigene NDA</t>
+          <t>eigene NDA; vor Unterzeichnung 22.07.</t>
         </is>
       </c>
       <c r="I19" s="25" t="n"/>
@@ -8724,7 +8739,7 @@
         </is>
       </c>
       <c r="E21" s="25" t="n">
-        <v>46235</v>
+        <v>46234</v>
       </c>
       <c r="F21" s="30" t="inlineStr">
         <is>
@@ -8736,7 +8751,11 @@
           <t>mittel</t>
         </is>
       </c>
-      <c r="H21" s="34" t="inlineStr"/>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>vor Lieferung 03.08.; 01.08. = Bundesfeier</t>
+        </is>
+      </c>
       <c r="I21" s="25" t="n"/>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Diagramm-Bugs behoben: Achsen-Namen, Prozente, Werte-Labels
Ursachen im Chart-XML gefunden und gefixt:
- Kategorien (Owner-Namen, Status) waren als numRef statt strRef
  gespeichert -> Excel zeigte keine Namen an der Kategorienachse
- Wertachse des Balken-Charts stand auf axPos 'l' statt 'b'
  -> keine Zahlen an der Achse
- Keine Datenbeschriftungen vorhanden -> jetzt Prozente im
  Status-Doughnut (showPercent) und Werte an den Balken (showVal)
- Achsen explizit sichtbar (delete=0) + tickLblPos nextTo

Verifier um 7 Chart-Checks erweitert (strRef, dLbls, Achsen, plotVisOnly);
alle Pruefungen PASS.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YMxj9pzhuMuXneYjMXFmRT
</commit_message>
<xml_diff>
--- a/Projektsteuerung_MiT-PWR-WIN-2026-001.xlsx
+++ b/Projektsteuerung_MiT-PWR-WIN-2026-001.xlsx
@@ -741,9 +741,9 @@
             </spPr>
           </dPt>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Dashboard'!$J$2:$J$6</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -751,6 +751,9 @@
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <showPercent val="1"/>
+        </dLbls>
         <firstSliceAng val="0"/>
         <holeSize val="55"/>
       </doughnutChart>
@@ -803,9 +806,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Dashboard'!$B$36:$B$45</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -813,6 +816,9 @@
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <showVal val="1"/>
+        </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -822,9 +828,11 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -833,10 +841,12 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <delete val="0"/>
+        <axPos val="b"/>
         <majorGridlines/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
@@ -932,8 +942,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Aenderungslog" displayName="Aenderungslog" ref="A1:E28" headerRowCount="1">
-  <autoFilter ref="A1:E28"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Aenderungslog" displayName="Aenderungslog" ref="A1:E29" headerRowCount="1">
+  <autoFilter ref="A1:E29"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Datum"/>
     <tableColumn id="2" name="Wer"/>
@@ -4483,7 +4493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4696,11 +4706,29 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="n"/>
-      <c r="B9" s="33" t="n"/>
-      <c r="C9" s="29" t="n"/>
-      <c r="D9" s="33" t="n"/>
-      <c r="E9" s="33" t="n"/>
+      <c r="A9" s="26" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B9" s="33" t="inlineStr">
+        <is>
+          <t>Burak Uecoez</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>Aenderung</t>
+        </is>
+      </c>
+      <c r="D9" s="33" t="inlineStr">
+        <is>
+          <t>Diagramm-Fixes: Owner-Namen an der Achse, Prozente im Status-Ring, Werte an den Balken, Wertachse unten.</t>
+        </is>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="26" t="n"/>
@@ -4835,14 +4863,21 @@
       <c r="D28" s="33" t="n"/>
       <c r="E28" s="33" t="n"/>
     </row>
+    <row r="29">
+      <c r="A29" s="26" t="n"/>
+      <c r="B29" s="33" t="n"/>
+      <c r="C29" s="29" t="n"/>
+      <c r="D29" s="33" t="n"/>
+      <c r="E29" s="33" t="n"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:C28">
+  <conditionalFormatting sqref="C2:C29">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="13">
       <formula>"Entscheid"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
+    <dataValidation sqref="C2:C29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungueltige Eingabe" error="Bitte einen Wert aus der Liste waehlen." prompt="Wert aus Dropdown waehlen" type="list">
       <formula1>"Aenderung,Entscheid"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>